<commit_message>
Added the Create Job Excel File and Login API Excel file in testng
</commit_message>
<xml_diff>
--- a/src/test/resources/testData/PhoenixTestData.xlsx
+++ b/src/test/resources/testData/PhoenixTestData.xlsx
@@ -5,10 +5,11 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="LoginTestData" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="CreateJobTestData" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -20,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="52">
   <si>
     <t xml:space="preserve">password</t>
   </si>
@@ -38,6 +39,144 @@
   </si>
   <si>
     <t xml:space="preserve">iamqc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mst_service_location_id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mst_platform_id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mst_warrenty_status_id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mst_oem_id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">customer__first_name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">customer__last_name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">customer__mobile_number</t>
+  </si>
+  <si>
+    <t xml:space="preserve">customer__mobile_number_alt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">customer__email_id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">customer__email_id_alt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">customer_address__flat_number</t>
+  </si>
+  <si>
+    <t xml:space="preserve">customer_address__apartment_name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">customer_address__street_name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">customer_address__landmark</t>
+  </si>
+  <si>
+    <t xml:space="preserve">customer_address__area</t>
+  </si>
+  <si>
+    <t xml:space="preserve">customer_address__pincode</t>
+  </si>
+  <si>
+    <t xml:space="preserve">customer_address__country</t>
+  </si>
+  <si>
+    <t xml:space="preserve">customer_address__state</t>
+  </si>
+  <si>
+    <t xml:space="preserve">customer_product__dop</t>
+  </si>
+  <si>
+    <t xml:space="preserve">customer_product__serial_number</t>
+  </si>
+  <si>
+    <t xml:space="preserve">customer_product__imei1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">customer_product__imei2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">customer_product__popurl</t>
+  </si>
+  <si>
+    <t xml:space="preserve">customer_product__product_id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">customer_product__mst_model_id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">problems__id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">problems__remark</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Talia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Goodwin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">396-547-0642</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Edwardo_Jaskolski@gmail.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hamburg 201</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Skilife</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Noida sector 126</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MG road</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Noida</t>
+  </si>
+  <si>
+    <t xml:space="preserve">India</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Uttar Pradesh</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-03-02T18:30:00.000Z</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13535678468600</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Battery Issue</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jatin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ajinkya</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Palak</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nancy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kajal</t>
   </si>
 </sst>
 </file>
@@ -126,7 +265,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -136,6 +275,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -383,4 +526,1145 @@
     <oddFooter>&amp;C&amp;"Helvetica Neue,Regular"&amp;12&amp;K000000&amp;P</oddFooter>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:AA558"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="3" width="21.54"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="3" width="15.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="3" width="21.75"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="3" width="11.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="3" width="20.24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="3" width="19.93"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="3" width="24.65"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="3" width="27.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="3" width="27.25"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="3" width="21.65"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="3" width="29.15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="3" width="33.36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="3" width="29.36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="3" width="26.65"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="3" width="22.44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="3" width="25.45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="3" width="25.15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="3" width="22.95"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="3" width="23.03"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="3" width="31.44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="21" style="3" width="23.45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="23" min="23" style="3" width="24.45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="24" min="24" style="3" width="28.07"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="25" min="25" style="3" width="30.85"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="V1" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="W1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="X1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="Y1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="Z1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="AA1" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="B2" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="C2" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="M2" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="N2" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="O2" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="P2" s="1" t="n">
+        <v>201303</v>
+      </c>
+      <c r="Q2" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="R2" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="S2" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="T2" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="U2" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="V2" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="W2" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="X2" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y2" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z2" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA2" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="B3" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="K3" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="L3" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="M3" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="N3" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="O3" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="P3" s="1" t="n">
+        <v>201303</v>
+      </c>
+      <c r="Q3" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="R3" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="S3" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="T3" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="U3" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="V3" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="W3" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="X3" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y3" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z3" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA3" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="B4" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="C4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="K4" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="L4" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="M4" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="N4" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="O4" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="P4" s="1" t="n">
+        <v>201303</v>
+      </c>
+      <c r="Q4" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="R4" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="S4" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="T4" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="U4" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="V4" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="W4" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="X4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA4" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="B5" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="C5" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="I5" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="K5" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="L5" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="M5" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="N5" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="O5" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="P5" s="1" t="n">
+        <v>201303</v>
+      </c>
+      <c r="Q5" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="R5" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="S5" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="T5" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="U5" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="V5" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="W5" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="X5" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y5" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z5" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA5" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="B6" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="C6" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="I6" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="K6" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="L6" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="M6" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="N6" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="O6" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="P6" s="1" t="n">
+        <v>201303</v>
+      </c>
+      <c r="Q6" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="R6" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="S6" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="T6" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="U6" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="V6" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="W6" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="X6" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y6" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z6" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA6" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="B7" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="C7" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="I7" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="K7" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="L7" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="M7" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="N7" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="O7" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="P7" s="1" t="n">
+        <v>201303</v>
+      </c>
+      <c r="Q7" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="R7" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="S7" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="T7" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="U7" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="V7" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="W7" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="X7" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y7" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z7" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA7" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="40" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="46" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="49" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="50" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="52" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="53" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="54" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="55" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="56" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="57" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="58" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="59" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="60" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="61" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="62" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="63" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="64" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="65" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="66" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="67" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="68" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="69" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="70" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="71" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="72" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="73" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="74" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="75" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="76" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="77" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="78" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="79" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="80" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="81" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="82" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="83" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="84" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="85" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="86" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="87" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="88" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="89" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="90" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="91" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="92" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="93" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="94" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="95" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="96" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="97" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="98" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="99" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="100" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="101" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="102" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="103" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="104" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="105" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="106" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="107" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="108" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="109" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="110" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="111" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="112" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="113" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="114" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="115" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="116" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="117" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="118" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="119" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="120" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="121" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="122" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="123" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="124" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="125" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="126" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="127" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="128" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="129" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="130" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="131" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="132" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="133" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="134" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="135" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="136" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="137" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="138" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="139" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="140" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="141" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="142" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="143" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="144" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="145" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="146" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="147" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="148" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="149" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="150" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="151" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="152" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="153" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="154" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="155" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="156" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="157" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="158" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="159" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="160" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="161" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="162" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="163" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="164" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="165" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="166" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="167" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="168" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="169" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="170" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="171" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="172" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="173" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="174" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="175" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="176" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="177" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="178" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="179" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="180" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="181" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="182" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="183" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="184" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="185" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="186" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="187" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="188" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="189" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="190" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="191" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="192" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="193" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="194" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="195" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="196" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="197" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="198" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="199" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="200" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="201" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="202" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="203" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="204" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="205" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="206" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="207" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="208" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="209" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="210" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="211" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="212" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="213" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="214" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="215" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="216" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="217" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="218" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="219" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="220" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="221" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="222" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="223" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="224" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="225" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="226" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="227" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="228" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="229" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="230" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="231" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="232" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="233" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="234" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="235" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="236" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="237" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="238" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="239" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="240" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="241" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="242" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="243" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="244" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="245" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="246" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="247" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="248" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="249" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="250" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="251" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="252" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="253" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="254" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="255" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="256" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="257" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="258" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="259" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="260" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="261" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="262" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="263" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="264" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="265" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="266" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="267" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="268" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="269" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="270" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="271" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="272" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="273" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="274" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="275" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="276" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="277" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="278" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="279" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="280" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="281" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="282" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="283" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="284" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="285" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="286" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="287" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="288" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="289" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="290" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="291" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="292" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="293" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="294" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="295" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="296" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="297" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="298" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="299" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="300" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="301" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="302" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="303" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="304" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="305" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="306" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="307" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="308" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="309" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="310" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="311" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="312" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="313" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="314" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="315" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="316" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="317" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="318" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="319" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="320" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="321" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="322" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="323" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="324" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="325" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="326" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="327" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="328" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="329" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="330" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="331" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="332" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="333" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="334" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="335" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="336" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="337" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="338" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="339" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="340" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="341" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="342" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="343" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="344" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="345" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="346" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="347" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="348" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="349" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="350" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="351" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="352" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="353" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="354" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="355" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="356" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="357" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="358" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="359" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="360" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="361" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="362" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="363" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="364" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="365" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="366" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="367" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="368" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="369" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="370" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="371" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="372" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="373" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="374" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="375" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="376" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="377" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="378" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="379" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="380" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="381" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="382" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="383" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="384" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="385" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="386" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="387" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="388" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="389" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="390" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="391" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="392" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="393" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="394" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="395" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="396" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="397" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="398" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="399" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="400" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="401" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="402" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="403" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="404" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="405" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="406" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="407" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="408" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="409" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="410" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="411" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="412" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="413" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="414" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="415" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="416" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="417" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="418" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="419" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="420" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="421" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="422" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="423" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="424" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="425" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="426" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="427" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="428" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="429" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="430" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="431" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="432" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="433" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="434" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="435" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="436" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="437" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="438" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="439" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="440" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="441" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="442" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="443" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="444" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="445" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="446" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="447" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="448" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="449" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="450" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="451" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="452" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="453" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="454" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="455" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="456" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="457" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="458" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="459" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="460" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="461" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="462" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="463" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="464" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="465" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="466" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="467" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="468" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="469" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="470" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="471" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="472" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="473" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="474" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="475" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="476" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="477" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="478" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="479" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="480" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="481" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="482" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="483" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="484" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="485" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="486" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="487" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="488" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="489" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="490" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="491" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="492" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="493" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="494" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="495" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="496" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="497" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="498" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="499" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="500" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="501" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="502" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="503" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="504" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="505" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="506" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="507" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="508" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="509" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="510" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="511" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="512" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="513" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="514" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="515" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="516" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="517" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="518" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="519" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="520" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="521" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="522" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="523" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="524" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="525" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="526" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="527" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="528" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="529" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="530" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="531" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="532" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="533" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="534" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="535" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="536" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="537" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="538" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="539" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="540" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="541" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="542" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="543" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="544" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="545" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="546" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="547" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="548" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="549" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="550" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="551" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="552" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="553" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="554" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="555" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="556" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="557" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="558" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>